<commit_message>
Correct Amazon reviewer name column fix
</commit_message>
<xml_diff>
--- a/exports/amazon-avaliacoes-budamix-2026-05-12.xlsx
+++ b/exports/amazon-avaliacoes-budamix-2026-05-12.xlsx
@@ -2105,10 +2105,10 @@
         <v>1</v>
       </c>
       <c r="K20" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L20" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M20" s="2" t="n">
         <v>1</v>
@@ -5960,10 +5960,14 @@
           <t>Kit 4 Potes De Vidro 640ml Tampa Hermético 4 Travas Vedação</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Maria Cecília Leite de Paiva Fernandes</t>
+        </is>
+      </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>perfil público parece conter frase, não nome</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -11606,7 +11610,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="9">
@@ -11616,7 +11620,7 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">

</xml_diff>